<commit_message>
fix: update excel header title from CareMetrics to FinSight to decouple project branding
</commit_message>
<xml_diff>
--- a/financial_analysis.xlsx
+++ b/financial_analysis.xlsx
@@ -558,7 +558,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="41" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
@@ -572,7 +572,7 @@
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>CareMetrics Financial Performance Summary</t>
+          <t>FinSight Financial Performance Summary</t>
         </is>
       </c>
     </row>

</xml_diff>